<commit_message>
feat: ship butcher unit and publishable lesson navigation
</commit_message>
<xml_diff>
--- a/outputs/019fbc71-4582-7bd0-b601-ad7557fe6608/v1-map-usability-pilot-toolkit.xlsx
+++ b/outputs/019fbc71-4582-7bd0-b601-ad7557fe6608/v1-map-usability-pilot-toolkit.xlsx
@@ -2,13 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R5a3bdbbc7ccd4f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总判定" sheetId="2" r:id="R0ff2a21922294b49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务脚本" sheetId="3" r:id="R7ac6cdba92e64abd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一轮观察" sheetId="4" r:id="R90faf675a1714ab7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第二轮观察" sheetId="5" r:id="R1f655f3375c04626"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="教师投屏" sheetId="6" r:id="Rf875c9ffe9eb47cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="7" r:id="Ra728e91f23a54f29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="1" r:id="R3734caeb601547e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总判定" sheetId="2" r:id="Rab6e3a1cef2943a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务脚本" sheetId="3" r:id="Rc6ac18a68e9f4b3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一轮观察" sheetId="4" r:id="Rbff36d3054b540ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第二轮观察" sheetId="5" r:id="Rfe373d051f67479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问题记录" sheetId="7" r:id="R6643d0874ead45b9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -295,7 +294,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -306,7 +305,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -317,7 +316,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -328,7 +327,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -339,7 +338,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -350,7 +349,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -361,7 +360,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -372,7 +371,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -383,7 +382,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -394,7 +393,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -405,7 +404,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF8E1B16"/>
         </x:patternFill>
       </x:fill>
@@ -416,7 +415,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEF5141"/>
         </x:patternFill>
       </x:fill>
@@ -427,7 +426,7 @@
         <x:color rgb="FF38281F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE1A6"/>
         </x:patternFill>
       </x:fill>
@@ -438,7 +437,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -449,7 +448,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -460,7 +459,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF8E1B16"/>
         </x:patternFill>
       </x:fill>
@@ -471,7 +470,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEF5141"/>
         </x:patternFill>
       </x:fill>
@@ -482,7 +481,7 @@
         <x:color rgb="FF38281F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE1A6"/>
         </x:patternFill>
       </x:fill>
@@ -493,7 +492,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -504,7 +503,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -515,7 +514,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF8E1B16"/>
         </x:patternFill>
       </x:fill>
@@ -526,7 +525,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEF5141"/>
         </x:patternFill>
       </x:fill>
@@ -537,7 +536,7 @@
         <x:color rgb="FF38281F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE1A6"/>
         </x:patternFill>
       </x:fill>
@@ -548,7 +547,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF8E1B16"/>
         </x:patternFill>
       </x:fill>
@@ -559,7 +558,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEF5141"/>
         </x:patternFill>
       </x:fill>
@@ -570,7 +569,7 @@
         <x:color rgb="FF38281F"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFE1A6"/>
         </x:patternFill>
       </x:fill>
@@ -581,7 +580,7 @@
         <x:color rgb="FF2F6D34"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE5F4E6"/>
         </x:patternFill>
       </x:fill>
@@ -592,7 +591,7 @@
         <x:color rgb="FFA52F26"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2DC"/>
         </x:patternFill>
       </x:fill>
@@ -638,28 +637,6 @@
     <x:tableColumn id="11" name="任务完成情况"/>
     <x:tableColumn id="12" name="最高严重度"/>
     <x:tableColumn id="13" name="观察备注（不要写姓名）"/>
-  </x:tableColumns>
-  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</x:table>
-</file>
-
-<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TeacherPresentationChecks" displayName="TeacherPresentationChecks" ref="A4:N9" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="14">
-    <x:tableColumn id="1" name="记录行"/>
-    <x:tableColumn id="2" name="日期"/>
-    <x:tableColumn id="3" name="平台类别"/>
-    <x:tableColumn id="4" name="全程无现场指导"/>
-    <x:tableColumn id="5" name="进入公开投屏"/>
-    <x:tableColumn id="6" name="进入/退出全屏"/>
-    <x:tableColumn id="7" name="播放/重播音频"/>
-    <x:tableColumn id="8" name="显示/隐藏提示"/>
-    <x:tableColumn id="9" name="上一步/下一步"/>
-    <x:tableColumn id="10" name="退出回课程"/>
-    <x:tableColumn id="11" name="独立完成"/>
-    <x:tableColumn id="12" name="总用时（秒）"/>
-    <x:tableColumn id="13" name="最高严重度"/>
-    <x:tableColumn id="14" name="观察备注"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -974,7 +951,7 @@
         <x:v>回答</x:v>
       </x:c>
       <x:c r="B5" s="26" t="str">
-        <x:v>孩子能否在 30 秒内独立找到推荐课程、区分可用与正在绘制地点、理解一次地图成长；教师能否无现场指导完成投屏。</x:v>
+        <x:v>孩子能否在 30 秒内独立找到推荐课程、区分可用与正在绘制地点、理解一次地图成长。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="40.5" customHeight="1">
@@ -1106,7 +1083,7 @@
         <x:v>判定</x:v>
       </x:c>
       <x:c r="C18" s="28" t="str">
-        <x:v>查看“汇总判定”；只有分母达标、第二轮四项比例均不低于 80%、教师通过且无未解决多数 P0/P1 才通过。</x:v>
+        <x:v>查看“汇总判定”；只有分母达标、第二轮四项比例均不低于 80%、且无未解决多数 P0/P1 才通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="22.5" customHeight="1">
@@ -1162,7 +1139,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
-        <x:v>多数使用者无法找到推荐课程、区分地点、理解成长、返回地图或使用投屏。</x:v>
+        <x:v>多数人无法找到课程、区分地点、理解成长或返回地图。</x:v>
       </x:c>
       <x:c r="C23" s="28" t="str">
         <x:v>本轮不通过，修复后重新验证。</x:v>
@@ -1462,113 +1439,72 @@
     </x:row>
     <x:row r="23" ht="22.5" customHeight="1">
       <x:c r="A23" s="11" t="str">
-        <x:v>教师投屏判定</x:v>
+        <x:v>阻断问题判定</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
-        <x:v>教师投屏判定</x:v>
+        <x:v>阻断问题判定</x:v>
       </x:c>
       <x:c r="C23" s="11" t="str">
-        <x:v>教师投屏判定</x:v>
+        <x:v>阻断问题判定</x:v>
       </x:c>
       <x:c r="D23" s="11" t="str">
-        <x:v>教师投屏判定</x:v>
+        <x:v>阻断问题判定</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="26" t="str">
-        <x:v>有效教师尝试（分母）</x:v>
+        <x:v>未验证的多数 P0/P1</x:v>
       </x:c>
       <x:c r="B24" s="26" t="n">
-        <x:f>COUNTIF('教师投屏'!$D$5:$D$9,"&lt;&gt;")</x:f>
+        <x:f>COUNTIFS('问题记录'!$F$5:$F$44,"P0",'问题记录'!$G$5:$G$44,"是",'问题记录'!$L$5:$L$44,"&lt;&gt;已验证")+COUNTIFS('问题记录'!$F$5:$F$44,"P1",'问题记录'!$G$5:$G$44,"是",'问题记录'!$L$5:$L$44,"&lt;&gt;已验证")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="28" t="str">
-        <x:v>无指导独立完成（分子）</x:v>
-      </x:c>
-      <x:c r="B25" s="28" t="n">
-        <x:f>COUNTIF('教师投屏'!$K$5:$K$9,"是")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="24" customHeight="1">
-      <x:c r="A26" s="28" t="str">
-        <x:v>教师门槛</x:v>
-      </x:c>
-      <x:c r="B26" s="28" t="str">
-        <x:f>IF(B24=0,"HUMAN_REQUIRED — 待执行",IF(B25=B24,"通过","不通过"))</x:f>
+        <x:v>问题门槛</x:v>
+      </x:c>
+      <x:c r="B25" s="28" t="str">
+        <x:f>IF(B24=0,"通过","不通过")</x:f>
+        <x:v>通过</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="22.5" customHeight="1">
+      <x:c r="A27" s="11" t="str">
+        <x:v>最终状态</x:v>
+      </x:c>
+      <x:c r="B27" s="11" t="str">
+        <x:v>最终状态</x:v>
+      </x:c>
+      <x:c r="C27" s="11" t="str">
+        <x:v>最终状态</x:v>
+      </x:c>
+      <x:c r="D27" s="11" t="str">
+        <x:v>最终状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="39" t="str">
+        <x:v>V1 地图试用判定</x:v>
+      </x:c>
+      <x:c r="B28" s="43" t="str">
+        <x:f>IF(OR(B12=0,C12=0),"HUMAN_REQUIRED — 待执行",IF(AND(B21="达标",C21="达标",C14&gt;=$B$5,C16&gt;=$B$5,C18&gt;=$B$5,C20&gt;=$B$5,B25="通过"),"通过","不通过"))</x:f>
         <x:v>HUMAN_REQUIRED — 待执行</x:v>
       </x:c>
-    </x:row>
-    <x:row r="28" ht="22.5" customHeight="1">
-      <x:c r="A28" s="11" t="str">
-        <x:v>阻断问题判定</x:v>
-      </x:c>
-      <x:c r="B28" s="11" t="str">
-        <x:v>阻断问题判定</x:v>
-      </x:c>
-      <x:c r="C28" s="11" t="str">
-        <x:v>阻断问题判定</x:v>
-      </x:c>
-      <x:c r="D28" s="11" t="str">
-        <x:v>阻断问题判定</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29" ht="24" customHeight="1">
-      <x:c r="A29" s="26" t="str">
-        <x:v>未验证的多数 P0/P1</x:v>
-      </x:c>
-      <x:c r="B29" s="26" t="n">
-        <x:f>COUNTIFS('问题记录'!$F$5:$F$44,"P0",'问题记录'!$G$5:$G$44,"是",'问题记录'!$L$5:$L$44,"&lt;&gt;已验证")+COUNTIFS('问题记录'!$F$5:$F$44,"P1",'问题记录'!$G$5:$G$44,"是",'问题记录'!$L$5:$L$44,"&lt;&gt;已验证")</x:f>
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30" ht="24" customHeight="1">
-      <x:c r="A30" s="28" t="str">
-        <x:v>问题门槛</x:v>
-      </x:c>
-      <x:c r="B30" s="28" t="str">
-        <x:f>IF(B29=0,"通过","不通过")</x:f>
-        <x:v>通过</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32" ht="22.5" customHeight="1">
-      <x:c r="A32" s="11" t="str">
-        <x:v>最终状态</x:v>
-      </x:c>
-      <x:c r="B32" s="11" t="str">
-        <x:v>最终状态</x:v>
-      </x:c>
-      <x:c r="C32" s="11" t="str">
-        <x:v>最终状态</x:v>
-      </x:c>
-      <x:c r="D32" s="11" t="str">
-        <x:v>最终状态</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="33">
-      <x:c r="A33" s="39" t="str">
-        <x:v>V1 地图试用判定</x:v>
-      </x:c>
-      <x:c r="B33" s="43" t="str">
-        <x:f>IF(OR(B12=0,C12=0,B24=0),"HUMAN_REQUIRED — 待执行",IF(AND(B21="达标",C21="达标",C14&gt;=$B$5,C16&gt;=$B$5,C18&gt;=$B$5,C20&gt;=$B$5,B26="通过",B30="通过"),"通过","不通过"))</x:f>
-        <x:v>HUMAN_REQUIRED — 待执行</x:v>
-      </x:c>
-      <x:c r="C33" s="43"/>
-      <x:c r="D33" s="43"/>
-    </x:row>
-    <x:row r="34" ht="31.5" customHeight="1">
-      <x:c r="A34" s="46" t="str">
+      <x:c r="C28" s="43"/>
+      <x:c r="D28" s="43"/>
+    </x:row>
+    <x:row r="29" ht="31.5" customHeight="1">
+      <x:c r="A29" s="46" t="str">
         <x:v>注意：通过只表示地图在本次机构试用中达到可理解、可操作门槛，不表示学习效果、留存或长期表现改善。</x:v>
       </x:c>
-      <x:c r="B34" s="46" t="str">
+      <x:c r="B29" s="46" t="str">
         <x:v>注意：通过只表示地图在本次机构试用中达到可理解、可操作门槛，不表示学习效果、留存或长期表现改善。</x:v>
       </x:c>
-      <x:c r="C34" s="46" t="str">
+      <x:c r="C29" s="46" t="str">
         <x:v>注意：通过只表示地图在本次机构试用中达到可理解、可操作门槛，不表示学习效果、留存或长期表现改善。</x:v>
       </x:c>
-      <x:c r="D34" s="46" t="str">
+      <x:c r="D29" s="46" t="str">
         <x:v>注意：通过只表示地图在本次机构试用中达到可理解、可操作门槛，不表示学习效果、留存或长期表现改善。</x:v>
       </x:c>
     </x:row>
@@ -1578,24 +1514,19 @@
     <x:mergeCell ref="A2:D2"/>
     <x:mergeCell ref="A4:D4"/>
     <x:mergeCell ref="A23:D23"/>
-    <x:mergeCell ref="A28:D28"/>
-    <x:mergeCell ref="A32:D32"/>
-    <x:mergeCell ref="B33:D33"/>
-    <x:mergeCell ref="A34:D34"/>
+    <x:mergeCell ref="A27:D27"/>
+    <x:mergeCell ref="B28:D28"/>
+    <x:mergeCell ref="A29:D29"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B21:C21">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="是"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="否"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B26:B26">
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="通过"/>
-    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="不通过"/>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B30:B30">
+  <x:conditionalFormatting sqref="B25:B25">
     <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="通过"/>
     <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="不通过"/>
   </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="B33:D33">
+  <x:conditionalFormatting sqref="B28:D28">
     <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="通过"/>
     <x:cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="不通过"/>
   </x:conditionalFormatting>
@@ -1854,92 +1785,75 @@
     </x:row>
     <x:row r="17" ht="49.5" customHeight="1">
       <x:c r="A17" s="28" t="str">
-        <x:v>教师检查</x:v>
+        <x:v>汇总</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>另请教师在无现场指导下打开公开投屏。</x:v>
+        <x:v>只查看“汇总判定”公式结果。</x:v>
       </x:c>
       <x:c r="C17" s="28" t="str">
-        <x:v>进入、全屏、音频、提示、前后步、退出。</x:v>
+        <x:v>不修改 80%、人数范围或严重度口径。</x:v>
       </x:c>
       <x:c r="D17" s="28" t="str">
-        <x:v>填“教师投屏”；不记录孩子画面。</x:v>
+        <x:v>保留空白/失败分母，不挑选成功样本。</x:v>
       </x:c>
       <x:c r="E17" s="28" t="str">
-        <x:v>任何多数阻塞 P0/P1 记入问题表。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="49.5" customHeight="1">
-      <x:c r="A18" s="28" t="str">
-        <x:v>汇总</x:v>
-      </x:c>
-      <x:c r="B18" s="28" t="str">
-        <x:v>只查看“汇总判定”公式结果。</x:v>
-      </x:c>
-      <x:c r="C18" s="28" t="str">
-        <x:v>不修改 80%、人数范围或严重度口径。</x:v>
-      </x:c>
-      <x:c r="D18" s="28" t="str">
-        <x:v>保留空白/失败分母，不挑选成功样本。</x:v>
-      </x:c>
-      <x:c r="E18" s="28" t="str">
         <x:v>没有完整人工证据时保持待执行。</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="22.5" customHeight="1">
-      <x:c r="A20" s="11" t="str">
+    <x:row r="19" ht="22.5" customHeight="1">
+      <x:c r="A19" s="11" t="str">
         <x:v>求助与观察口径</x:v>
       </x:c>
-      <x:c r="B20" s="11" t="str">
+      <x:c r="B19" s="11" t="str">
         <x:v>求助与观察口径</x:v>
       </x:c>
-      <x:c r="C20" s="11" t="str">
+      <x:c r="C19" s="11" t="str">
         <x:v>求助与观察口径</x:v>
       </x:c>
-      <x:c r="D20" s="11" t="str">
+      <x:c r="D19" s="11" t="str">
         <x:v>求助与观察口径</x:v>
       </x:c>
-      <x:c r="E20" s="11" t="str">
+      <x:c r="E19" s="11" t="str">
         <x:v>求助与观察口径</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="33" customHeight="1">
-      <x:c r="A21" s="33" t="str">
+    <x:row r="20" ht="33" customHeight="1">
+      <x:c r="A20" s="33" t="str">
         <x:v>情况</x:v>
       </x:c>
-      <x:c r="B21" s="33" t="str">
+      <x:c r="B20" s="33" t="str">
         <x:v>统一处理</x:v>
       </x:c>
     </x:row>
+    <x:row r="21" ht="40.5" customHeight="1">
+      <x:c r="A21" s="26" t="str">
+        <x:v>孩子问“点哪里”</x:v>
+      </x:c>
+      <x:c r="B21" s="26" t="str">
+        <x:v>先记录当前用时和失败点，再给一个最小提示；求助次数 +1。</x:v>
+      </x:c>
+    </x:row>
     <x:row r="22" ht="40.5" customHeight="1">
-      <x:c r="A22" s="26" t="str">
-        <x:v>孩子问“点哪里”</x:v>
-      </x:c>
-      <x:c r="B22" s="26" t="str">
-        <x:v>先记录当前用时和失败点，再给一个最小提示；求助次数 +1。</x:v>
+      <x:c r="A22" s="28" t="str">
+        <x:v>超过 30 秒</x:v>
+      </x:c>
+      <x:c r="B22" s="28" t="str">
+        <x:v>记录实际秒数和“否”，随后可以帮助孩子继续完成其余任务。</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="40.5" customHeight="1">
       <x:c r="A23" s="28" t="str">
-        <x:v>超过 30 秒</x:v>
+        <x:v>孩子用颜色区分地点</x:v>
       </x:c>
       <x:c r="B23" s="28" t="str">
-        <x:v>记录实际秒数和“否”，随后可以帮助孩子继续完成其余任务。</x:v>
+        <x:v>追问“除了颜色，你还看到了什么？”；必须说出文字/图形状态才算通过。</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="40.5" customHeight="1">
       <x:c r="A24" s="28" t="str">
-        <x:v>孩子用颜色区分地点</x:v>
+        <x:v>孩子说“变漂亮了”</x:v>
       </x:c>
       <x:c r="B24" s="28" t="str">
-        <x:v>追问“除了颜色，你还看到了什么？”；必须说出文字/图形状态才算通过。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="40.5" customHeight="1">
-      <x:c r="A25" s="28" t="str">
-        <x:v>孩子说“变漂亮了”</x:v>
-      </x:c>
-      <x:c r="B25" s="28" t="str">
         <x:v>追问“哪里多了什么？”；能指出新增地标部件才算理解成长。</x:v>
       </x:c>
     </x:row>
@@ -1949,7 +1863,7 @@
     <x:mergeCell ref="A2:E2"/>
     <x:mergeCell ref="A4:E4"/>
     <x:mergeCell ref="A12:E12"/>
-    <x:mergeCell ref="A20:E20"/>
+    <x:mergeCell ref="A19:E19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2309,7 +2223,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4a6932883394eda"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40898af2b6424206"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3130,313 +3044,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R060d44022cd646f8"/>
-  </x:tableParts>
-</x:worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheetFormatPr defaultRowHeight="15"/>
-  <x:cols>
-    <x:col min="1" max="1" width="6.440000057220459" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="13.109999656677246" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="11.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="9.779999732971191" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="25.559999465942383" hidden="0" customWidth="1"/>
-  </x:cols>
-  <x:sheetData>
-    <x:row r="1" ht="33" customHeight="1">
-      <x:c r="A1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="C1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="D1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="E1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="F1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="G1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="H1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="I1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="J1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="K1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="L1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="M1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-      <x:c r="N1" s="4" t="str">
-        <x:v>教师公开投屏检查</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" ht="31.5" customHeight="1">
-      <x:c r="A2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="B2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="C2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="D2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="E2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="F2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="G2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="H2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="I2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="J2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="K2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="L2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="M2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-      <x:c r="N2" s="8" t="str">
-        <x:v>教师在没有现场指导、无需账号的条件下独立完成。记录操作结果，不记录课堂中的儿童画面或身份。</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="39" customHeight="1">
-      <x:c r="A4" s="33" t="str">
-        <x:v>记录行</x:v>
-      </x:c>
-      <x:c r="B4" s="33" t="str">
-        <x:v>日期</x:v>
-      </x:c>
-      <x:c r="C4" s="33" t="str">
-        <x:v>平台类别</x:v>
-      </x:c>
-      <x:c r="D4" s="33" t="str">
-        <x:v>全程无现场指导</x:v>
-      </x:c>
-      <x:c r="E4" s="33" t="str">
-        <x:v>进入公开投屏</x:v>
-      </x:c>
-      <x:c r="F4" s="33" t="str">
-        <x:v>进入/退出全屏</x:v>
-      </x:c>
-      <x:c r="G4" s="33" t="str">
-        <x:v>播放/重播音频</x:v>
-      </x:c>
-      <x:c r="H4" s="33" t="str">
-        <x:v>显示/隐藏提示</x:v>
-      </x:c>
-      <x:c r="I4" s="33" t="str">
-        <x:v>上一步/下一步</x:v>
-      </x:c>
-      <x:c r="J4" s="33" t="str">
-        <x:v>退出回课程</x:v>
-      </x:c>
-      <x:c r="K4" s="33" t="str">
-        <x:v>独立完成</x:v>
-      </x:c>
-      <x:c r="L4" s="33" t="str">
-        <x:v>总用时（秒）</x:v>
-      </x:c>
-      <x:c r="M4" s="33" t="str">
-        <x:v>最高严重度</x:v>
-      </x:c>
-      <x:c r="N4" s="33" t="str">
-        <x:v>观察备注</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="26" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B5" s="53"/>
-      <x:c r="C5" s="26"/>
-      <x:c r="D5" s="26"/>
-      <x:c r="E5" s="26"/>
-      <x:c r="F5" s="26"/>
-      <x:c r="G5" s="26"/>
-      <x:c r="H5" s="26"/>
-      <x:c r="I5" s="26"/>
-      <x:c r="J5" s="26"/>
-      <x:c r="K5" s="57" t="str">
-        <x:f>IF(D5="","",IF(AND(D5="是",E5="是",F5="是",G5="是",H5="是",I5="是",J5="是"),"是","否"))</x:f>
-      </x:c>
-      <x:c r="L5" s="55"/>
-      <x:c r="M5" s="26"/>
-      <x:c r="N5" s="26"/>
-    </x:row>
-    <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="28" t="n">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B6" s="54"/>
-      <x:c r="C6" s="28"/>
-      <x:c r="D6" s="28"/>
-      <x:c r="E6" s="28"/>
-      <x:c r="F6" s="28"/>
-      <x:c r="G6" s="28"/>
-      <x:c r="H6" s="28"/>
-      <x:c r="I6" s="28"/>
-      <x:c r="J6" s="28"/>
-      <x:c r="K6" s="58" t="str">
-        <x:f>IF(D6="","",IF(AND(D6="是",E6="是",F6="是",G6="是",H6="是",I6="是",J6="是"),"是","否"))</x:f>
-      </x:c>
-      <x:c r="L6" s="56"/>
-      <x:c r="M6" s="28"/>
-      <x:c r="N6" s="28"/>
-    </x:row>
-    <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="28" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B7" s="54"/>
-      <x:c r="C7" s="28"/>
-      <x:c r="D7" s="28"/>
-      <x:c r="E7" s="28"/>
-      <x:c r="F7" s="28"/>
-      <x:c r="G7" s="28"/>
-      <x:c r="H7" s="28"/>
-      <x:c r="I7" s="28"/>
-      <x:c r="J7" s="28"/>
-      <x:c r="K7" s="58" t="str">
-        <x:f>IF(D7="","",IF(AND(D7="是",E7="是",F7="是",G7="是",H7="是",I7="是",J7="是"),"是","否"))</x:f>
-      </x:c>
-      <x:c r="L7" s="56"/>
-      <x:c r="M7" s="28"/>
-      <x:c r="N7" s="28"/>
-    </x:row>
-    <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="28" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="B8" s="54"/>
-      <x:c r="C8" s="28"/>
-      <x:c r="D8" s="28"/>
-      <x:c r="E8" s="28"/>
-      <x:c r="F8" s="28"/>
-      <x:c r="G8" s="28"/>
-      <x:c r="H8" s="28"/>
-      <x:c r="I8" s="28"/>
-      <x:c r="J8" s="28"/>
-      <x:c r="K8" s="58" t="str">
-        <x:f>IF(D8="","",IF(AND(D8="是",E8="是",F8="是",G8="是",H8="是",I8="是",J8="是"),"是","否"))</x:f>
-      </x:c>
-      <x:c r="L8" s="56"/>
-      <x:c r="M8" s="28"/>
-      <x:c r="N8" s="28"/>
-    </x:row>
-    <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="28" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B9" s="54"/>
-      <x:c r="C9" s="28"/>
-      <x:c r="D9" s="28"/>
-      <x:c r="E9" s="28"/>
-      <x:c r="F9" s="28"/>
-      <x:c r="G9" s="28"/>
-      <x:c r="H9" s="28"/>
-      <x:c r="I9" s="28"/>
-      <x:c r="J9" s="28"/>
-      <x:c r="K9" s="58" t="str">
-        <x:f>IF(D9="","",IF(AND(D9="是",E9="是",F9="是",G9="是",H9="是",I9="是",J9="是"),"是","否"))</x:f>
-      </x:c>
-      <x:c r="L9" s="56"/>
-      <x:c r="M9" s="28"/>
-      <x:c r="N9" s="28"/>
-    </x:row>
-  </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:N1"/>
-    <x:mergeCell ref="A2:N2"/>
-  </x:mergeCells>
-  <x:conditionalFormatting sqref="D5:K9">
-    <x:cfRule type="containsText" dxfId="18" priority="1" operator="containsText" text="是"/>
-    <x:cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="否"/>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="M5:M9">
-    <x:cfRule type="containsText" dxfId="20" priority="3" operator="containsText" text="P0"/>
-    <x:cfRule type="containsText" dxfId="21" priority="4" operator="containsText" text="P1"/>
-    <x:cfRule type="containsText" dxfId="22" priority="5" operator="containsText" text="P2"/>
-  </x:conditionalFormatting>
-  <x:dataValidations count="10">
-    <x:dataValidation type="list" sqref="C5:C9">
-      <x:formula1>"微信内置浏览器,iPhone Safari,Android Chromium,平板,桌面投屏"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="D5:D9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="E5:E9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="F5:F9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="G5:G9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="H5:H9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="I5:I9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="J5:J9">
-      <x:formula1>"是,否"</x:formula1>
-    </x:dataValidation>
-    <x:dataValidation type="whole" operator="between" sqref="L5:L9">
-      <x:formula1>0</x:formula1>
-      <x:formula2>1800</x:formula2>
-    </x:dataValidation>
-    <x:dataValidation type="list" sqref="M5:M9">
-      <x:formula1>"无,P0,P1,P2"</x:formula1>
-    </x:dataValidation>
-  </x:dataValidations>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re91d73dadbd441a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78f90637b5ac4f10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4279,10 +3887,10 @@
   </x:conditionalFormatting>
   <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="B5:B44">
-      <x:formula1>"第一轮,第二轮,教师投屏"</x:formula1>
+      <x:formula1>"第一轮,第二轮"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="E5:E44">
-      <x:formula1>"微信内置浏览器,iPhone Safari,Android Chromium,平板,桌面投屏,其他演示设备"</x:formula1>
+      <x:formula1>"微信内置浏览器,iPhone Safari,Android Chromium,平板,桌面浏览器,其他演示设备"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F5:F44">
       <x:formula1>"P0,P1,P2"</x:formula1>
@@ -4296,7 +3904,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R203931e3cdd746cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10a6773fe91845b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>